<commit_message>
docs(ae2): informe v3 con dependencias entre tareas y marco justificado; bitacora y registro de corridas actualizados
Agrega la tabla de dependencias y la ruta sin margen (V.4), la justificacion del marco agil (V.1), la lectura del prototipo en el mapa de competencia (IV.4) y los enlaces finales. La bitacora retira la afirmacion del clonado del 29/09 y declara el uso 7 de IA.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
+++ b/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="118">
   <si>
     <t>Registro de corridas de GitHub Actions · ThiagoML22/motelOS-pfg</t>
   </si>
   <si>
-    <t>Exportado el 05/10/2026 22:10 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
+    <t>Exportado el 05/10/2026 23:01 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
   </si>
   <si>
     <t>N.º</t>
@@ -346,10 +346,28 @@
     <t>Merge v1.2: RNF-08 (patente separada y depurada a las 24 h) y rol mot…</t>
   </si>
   <si>
+    <t>05/10/2026 22:15:35</t>
+  </si>
+  <si>
+    <t>8498d3a</t>
+  </si>
+  <si>
+    <t>docs(ae2): documentos de la Ventana de Mejora (informe v3, catalogo v…</t>
+  </si>
+  <si>
+    <t>05/10/2026 22:57:11</t>
+  </si>
+  <si>
+    <t>d9fec30</t>
+  </si>
+  <si>
+    <t>docs: la declaracion de IA del README incluye el codigo de la v1.2</t>
+  </si>
+  <si>
     <t>Resumen</t>
   </si>
   <si>
-    <t>31 corridas: 22 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
+    <t>33 corridas: 24 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
   </si>
 </sst>
 </file>
@@ -759,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1469,23 +1487,65 @@
         <v>109</v>
       </c>
     </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="4">
+        <v>32</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="3" t="s">
-        <v>110</v>
+      <c r="A37" s="4">
+        <v>33</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C37" s="4"/>
+        <v>113</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>114</v>
+      </c>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="E37" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(ae2): requisitos validados por la gerencia (acta del 06/10), prueba de clonado sobre la v1.2 y datos del negocio confirmados
Los 22 requisitos quedan validados; la tarifa, el plazo de 24 h de la patente, el arqueo en la guardia que cobra y la exclusion de datos del cliente estan aprobados. La perdida mensual de $380.000 la confirma la gerencia por escrito. El escaneo firmado no se publica en el repositorio.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
+++ b/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="124">
   <si>
     <t>Registro de corridas de GitHub Actions · ThiagoML22/motelOS-pfg</t>
   </si>
   <si>
-    <t>Exportado el 05/10/2026 23:01 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
+    <t>Exportado el 07/10/2026 21:25 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
   </si>
   <si>
     <t>N.º</t>
@@ -364,10 +364,28 @@
     <t>docs: la declaracion de IA del README incluye el codigo de la v1.2</t>
   </si>
   <si>
+    <t>05/10/2026 23:04:36</t>
+  </si>
+  <si>
+    <t>bb0a13b</t>
+  </si>
+  <si>
+    <t>docs(ae2): informe v3 con dependencias entre tareas y marco justifica…</t>
+  </si>
+  <si>
+    <t>07/10/2026 20:55:44</t>
+  </si>
+  <si>
+    <t>27892f3</t>
+  </si>
+  <si>
+    <t>docs(ae2): correcciones de la AE1 reflejan que la AE1 ya estaba cargada</t>
+  </si>
+  <si>
     <t>Resumen</t>
   </si>
   <si>
-    <t>33 corridas: 24 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
+    <t>35 corridas: 26 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
   </si>
 </sst>
 </file>
@@ -777,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1529,23 +1547,65 @@
         <v>115</v>
       </c>
     </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="4">
+        <v>34</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D38" s="4"/>
+      <c r="E38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="3" t="s">
-        <v>116</v>
+      <c r="A39" s="4">
+        <v>35</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C39" s="4"/>
+        <v>119</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>120</v>
+      </c>
       <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
+      <c r="E39" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B41:G41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(ae2): respuestas 1 y 8 del Bloque A cerradas; todos los commits declarados con Claude Code
La declaracion de IA del README y de la bitacora dice que todos los commits del prototipo se realizaron con Claude Code. Se retiran los pendientes que ya no corresponden y se declaran como propuesta del autor el procedimiento ante un corte de internet y la resolucion minima del monitor.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
+++ b/docs/AE2/20261004_Registro_corridas_Actions_motelOS.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="130">
   <si>
     <t>Registro de corridas de GitHub Actions · ThiagoML22/motelOS-pfg</t>
   </si>
   <si>
-    <t>Exportado el 07/10/2026 21:25 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
+    <t>Exportado el 07/10/2026 22:17 (hora de Argentina) desde la API pública de GitHub. La hora de cada corrida es la de su creación, convertida de UTC a UTC-3.</t>
   </si>
   <si>
     <t>N.º</t>
@@ -382,10 +382,28 @@
     <t>docs(ae2): correcciones de la AE1 reflejan que la AE1 ya estaba cargada</t>
   </si>
   <si>
+    <t>07/10/2026 21:27:35</t>
+  </si>
+  <si>
+    <t>36d8638</t>
+  </si>
+  <si>
+    <t>docs(ae2): requisitos validados por la gerencia (acta del 06/10), pru…</t>
+  </si>
+  <si>
+    <t>07/10/2026 21:52:34</t>
+  </si>
+  <si>
+    <t>6c58de7</t>
+  </si>
+  <si>
+    <t>docs(ae2): Instrumento 27 con la exclusion de datos filiatorios validada</t>
+  </si>
+  <si>
     <t>Resumen</t>
   </si>
   <si>
-    <t>35 corridas: 26 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
+    <t>37 corridas: 28 exitosas y 9 fallidas. Las fallidas están entre las diez primeras (25 al 28/09/2026); desde la n.º 11 todas pasan.</t>
   </si>
 </sst>
 </file>
@@ -795,7 +813,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1589,23 +1607,65 @@
         <v>121</v>
       </c>
     </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="4">
+        <v>36</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="E40" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="3" t="s">
-        <v>122</v>
+      <c r="A41" s="4">
+        <v>37</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C41" s="4"/>
+        <v>125</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
+      <c r="E41" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B43:G43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>